<commit_message>
Add timestamped transcript support for WOOM subpages
</commit_message>
<xml_diff>
--- a/WOOM Archive Inputs.xlsx
+++ b/WOOM Archive Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Creative\Podcasts\Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E57926D-0E7C-4BEB-AF6C-BF29D009AD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E34D6F-2ACB-4A1D-92F0-932BD8BB6AC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF7F1007-203D-4DE6-BF2A-5A27FA14567C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DF7F1007-203D-4DE6-BF2A-5A27FA14567C}"/>
   </bookViews>
   <sheets>
     <sheet name="WOOM Archive" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="257">
   <si>
     <t>youtube_link</t>
   </si>
@@ -7611,7 +7611,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -7620,7 +7620,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -7650,10 +7649,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7993,7 +7988,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>178</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -8001,653 +7996,653 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" t="s">
         <v>107</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>108</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>109</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" t="s">
         <v>110</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" t="s">
         <v>111</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" t="s">
         <v>112</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" t="s">
         <v>113</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" t="s">
         <v>114</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" t="s">
         <v>115</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" t="s">
         <v>116</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" t="s">
         <v>117</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" t="s">
         <v>118</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" t="s">
         <v>119</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" t="s">
         <v>120</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="E15" s="6"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" t="s">
         <v>121</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="E16" s="6"/>
+      <c r="E16" s="5"/>
     </row>
     <row r="17" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" t="s">
         <v>122</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="5" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" t="s">
         <v>123</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="5" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" t="s">
         <v>124</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="5" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" t="s">
         <v>125</v>
       </c>
       <c r="B20" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="5" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" t="s">
         <v>126</v>
       </c>
       <c r="B21" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="E21" s="6"/>
+      <c r="E21" s="5"/>
     </row>
     <row r="22" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" t="s">
         <v>127</v>
       </c>
       <c r="B22" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="5" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" t="s">
         <v>128</v>
       </c>
       <c r="B23" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="5" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" t="s">
         <v>129</v>
       </c>
       <c r="B24" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="5" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" t="s">
         <v>130</v>
       </c>
       <c r="B25" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="E25" s="6"/>
+      <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="A26" t="s">
         <v>131</v>
       </c>
       <c r="B26" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="5" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="A27" t="s">
         <v>132</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="E27" s="6"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="A28" t="s">
         <v>133</v>
       </c>
       <c r="B28" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="5" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="A29" t="s">
         <v>134</v>
       </c>
       <c r="B29" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="5" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+      <c r="A30" t="s">
         <v>135</v>
       </c>
       <c r="B30" t="s">
         <v>31</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="5" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="A31" t="s">
         <v>136</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="5" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="A32" t="s">
         <v>137</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+      <c r="A33" t="s">
         <v>138</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="5" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+      <c r="A34" t="s">
         <v>139</v>
       </c>
       <c r="B34" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="5" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+      <c r="A35" t="s">
         <v>140</v>
       </c>
       <c r="B35" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="5" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+      <c r="A36" t="s">
         <v>141</v>
       </c>
       <c r="B36" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="5" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
+      <c r="A37" t="s">
         <v>142</v>
       </c>
       <c r="B37" t="s">
         <v>38</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="5" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+      <c r="A38" t="s">
         <v>143</v>
       </c>
       <c r="B38" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E38" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="A39" t="s">
         <v>144</v>
       </c>
       <c r="B39" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="E39" s="6"/>
+      <c r="E39" s="5"/>
     </row>
     <row r="40" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+      <c r="A40" t="s">
         <v>145</v>
       </c>
       <c r="B40" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="E40" s="6"/>
+      <c r="E40" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E40" xr:uid="{77C17E25-847F-43D6-AEDB-CD2A150F451C}"/>
@@ -8660,436 +8655,557 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{214257A5-E9A4-4538-96DF-EBCBFEE3F0D1}">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="66.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.28515625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>43</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>119</v>
+      </c>
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" t="s">
         <v>18</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>124</v>
+      </c>
+      <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B20" t="s">
         <v>21</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>126</v>
+      </c>
+      <c r="B21" t="s">
         <v>22</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" t="s">
         <v>23</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" t="s">
         <v>25</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" t="s">
         <v>24</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" t="s">
         <v>26</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="D25" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" t="s">
         <v>27</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="D26" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" t="s">
         <v>28</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" t="s">
         <v>29</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>68</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="D28" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>134</v>
+      </c>
+      <c r="B29" t="s">
         <v>30</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>69</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>135</v>
+      </c>
+      <c r="B30" t="s">
         <v>31</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="D30" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>136</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" t="s">
+        <v>32</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" t="s">
+        <v>33</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>138</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" t="s">
+        <v>34</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="B34" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>140</v>
       </c>
       <c r="B35" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="B36" t="s">
         <v>37</v>
       </c>
+      <c r="C36" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>142</v>
       </c>
       <c r="B37" t="s">
         <v>38</v>
       </c>
+      <c r="C37" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>143</v>
       </c>
       <c r="B38" t="s">
         <v>39</v>
       </c>
+      <c r="C38" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>144</v>
       </c>
       <c r="B39" t="s">
         <v>40</v>
       </c>
+      <c r="C39" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>145</v>
+      </c>
+      <c r="B40" t="s">
         <v>41</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploy updated spreadsheets with preserved top back buttons and mobile header toggle
</commit_message>
<xml_diff>
--- a/WOOM Archive Inputs.xlsx
+++ b/WOOM Archive Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Creative\Podcasts\Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE37E48-003A-4107-AB1F-4D2DCBCFB419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77F0F4C-3227-4039-B16A-105F00E45DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF7F1007-203D-4DE6-BF2A-5A27FA14567C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF7F1007-203D-4DE6-BF2A-5A27FA14567C}"/>
   </bookViews>
   <sheets>
     <sheet name="WOOM Archive" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="267">
   <si>
     <t>youtube_link</t>
   </si>
@@ -9005,48 +9005,6 @@
     <t>09.08.26</t>
   </si>
   <si>
-    <t>Topics Covered
-• DaBaby's Charlotte food truck, IG restaurant culture, and whether any food is worth a three-hour wait 
-• Funny childhood decisions that probably terrified their parents 
-• Running away as a joke, dangerous sledding, trampoline stunts, stair surfing, and neighborhood mischief 
-• Family traditions that are disappearing and who is responsible for preserving them 
-• Millennials inheriting the responsibilities once handled by parents, grandparents, aunts, and uncles 
-• Analysis paralysis versus taking action and building momentum through consistency 
-• Podcasting, audience-building, and becoming part of someone's routine 
-• Posting content online, social media anxiety, and worrying about public judgment 
-• Whether hobbies should become businesses or sources of income 
-• Influencer culture, authenticity, and the dangers of turning everything into content 
-Best Questions
-• Is there any restaurant worth standing in line three hours to eat at? 
-• What is the funniest thing you did as a child that terrified your parents? 
-• Which family traditions are actually worth preserving? 
-• Why do talented people get stuck while less-talented people succeed? 
-• Should hobbies be monetized? 
-• At what point does content creation stop being fun and start becoming work?
-Best Observations
-• Many traditions disappear not because older generations stop caring, but because younger generations never pick up the baton. 
-• Consistency often beats talent because people become part of their audience's routine. 
-• Most creators are terrible judges of what audiences will actually connect with. 
-• An unfinished project seen by people is usually more valuable than a perfect project that never leaves the hard drive. 
-• Social media rewards authenticity but simultaneously pressures creators toward performance. 
-• Many hobbies become less enjoyable when every moment is optimized for engagement and monetization. 
-Best Debate
-Should Hobbies Make Money?
-Jordan argued that there is nothing wrong with earning money from something you already love doing and that monetization can be a blessing when it happens naturally. Darius countered that commercialization can slowly drain enjoyment from a hobby and pointed to influencers who clearly no longer enjoy the content they create but continue because it has become their job.
-Themes
-• Childhood memories
-• Family traditions
-• Adulthood
-• Community responsibility
-• Consistency
-• Creativity
-• Podcasting
-• Social media
-• Content creation
-• Monetization
-• Influencer culture</t>
-  </si>
-  <si>
     <t>Transcript
 00:00:00 Darius
 We have to grab the baton. Traditions are dying out because we keep expecting the grownups to do it. But we're the grownups.
@@ -9333,6 +9291,63 @@
   </si>
   <si>
     <t>Grab the Baton: Cookouts, Childhood Chaos &amp; Creative Discipline</t>
+  </si>
+  <si>
+    <t>&lt;section class="show-notes-highlights"&gt;
+  &lt;h2&gt;Show Notes &amp;amp; Highlights&lt;/h2&gt;
+  &lt;h3&gt;Topics Covered&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;DaBaby&amp;#39;s Charlotte food truck, IG restaurant culture, and whether any food is worth a three-hour wait&lt;/li&gt;
+    &lt;li&gt;Funny childhood decisions that probably terrified their parents&lt;/li&gt;
+    &lt;li&gt;Running away as a joke, dangerous sledding, trampoline stunts, stair surfing, and neighborhood mischief&lt;/li&gt;
+    &lt;li&gt;Family traditions that are disappearing and who is responsible for preserving them&lt;/li&gt;
+    &lt;li&gt;Millennials inheriting the responsibilities once handled by parents, grandparents, aunts, and uncles&lt;/li&gt;
+    &lt;li&gt;Analysis paralysis versus taking action and building momentum through consistency&lt;/li&gt;
+    &lt;li&gt;Podcasting, audience-building, and becoming part of someone&amp;#39;s routine&lt;/li&gt;
+    &lt;li&gt;Posting content online, social media anxiety, and worrying about public judgment&lt;/li&gt;
+    &lt;li&gt;Whether hobbies should become businesses or sources of income&lt;/li&gt;
+    &lt;li&gt;Influencer culture, authenticity, and the dangers of turning everything into content&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Best Questions&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Is there any restaurant worth standing in line three hours to eat at?&lt;/li&gt;
+    &lt;li&gt;What is the funniest thing you did as a child that terrified your parents?&lt;/li&gt;
+    &lt;li&gt;Which family traditions are actually worth preserving?&lt;/li&gt;
+    &lt;li&gt;Why do talented people get stuck while less-talented people succeed?&lt;/li&gt;
+    &lt;li&gt;Should hobbies be monetized?&lt;/li&gt;
+    &lt;li&gt;At what point does content creation stop being fun and start becoming work?&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Best Observations&lt;/h3&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Many traditions disappear not because older generations stop caring, but because younger generations never pick up the baton.&lt;/li&gt;
+    &lt;li&gt;Consistency often beats talent because people become part of their audience&amp;#39;s routine.&lt;/li&gt;
+    &lt;li&gt;Most creators are terrible judges of what audiences will actually connect with.&lt;/li&gt;
+    &lt;li&gt;An unfinished project seen by people is usually more valuable than a perfect project that never leaves the hard drive.&lt;/li&gt;
+    &lt;li&gt;Social media rewards authenticity but simultaneously pressures creators toward performance.&lt;/li&gt;
+    &lt;li&gt;Many hobbies become less enjoyable when every moment is optimized for engagement and monetization.&lt;/li&gt;
+  &lt;/ul&gt;
+  &lt;h3&gt;Best Debate&lt;/h3&gt;
+  &lt;p&gt;Should Hobbies Make Money? Jordan argued that there is nothing wrong with earning money from something you already love doing and that monetization can be a blessing when it happens naturally. Darius countered that commercialization can slowly drain enjoyment from a hobby and pointed to influencers who clearly no longer enjoy the content they create but continue because it has become their job.&lt;/p&gt;
+  &lt;div class="major-themes"&gt;
+    &lt;h3&gt;Major Themes&lt;/h3&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Childhood memories&lt;/li&gt;
+      &lt;li&gt;Family traditions&lt;/li&gt;
+      &lt;li&gt;Adulthood&lt;/li&gt;
+      &lt;li&gt;Community responsibility&lt;/li&gt;
+      &lt;li&gt;Consistency&lt;/li&gt;
+      &lt;li&gt;Creativity&lt;/li&gt;
+      &lt;li&gt;Podcasting&lt;/li&gt;
+      &lt;li&gt;Social media&lt;/li&gt;
+      &lt;li&gt;Content creation&lt;/li&gt;
+      &lt;li&gt;Monetization&lt;/li&gt;
+      &lt;li&gt;Influencer culture&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/div&gt;
+&lt;/section&gt;</t>
+  </si>
+  <si>
+    <t>2026-09-08</t>
   </si>
 </sst>
 </file>
@@ -10458,16 +10473,16 @@
     </row>
     <row r="41" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B41" t="s">
         <v>262</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="E41" s="5"/>
     </row>
@@ -11054,16 +11069,16 @@
     </row>
     <row r="41" spans="1:4" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B41" t="s">
         <v>262</v>
       </c>
-      <c r="C41" t="s">
-        <v>262</v>
+      <c r="C41" s="7" t="s">
+        <v>266</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>